<commit_message>
Contratos: empresa (Charão / LuS) e tipo de contrato
- Configurações > Tipos de contrato (lista própria, já com 9 tipos)
- Contrato com empresa e tipo; boletim sai com o logo e o nome da empresa
- Painel inteiro filtra por empresa e tipo (inclui 'Sem tipo' para revisar)
- Contratos existentes: tipo pelo início do nome (uma vez na subida)
- Importar BMs: empresa pela conta '(LUS)' e tipo pelo nome; na prévia dá para ajustar,
  inclusive dos contratos já importados (empresa escolhida à mão não muda)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/fixtures/recebimentos-exemplo-baixa.xlsx
+++ b/scripts/fixtures/recebimentos-exemplo-baixa.xlsx
@@ -863,13 +863,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFC8F281-5893-4802-B075-160EBB91035C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3F51F24-116C-4AFF-8F83-B73AE5BB373F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0271910-A1AA-4E53-B29E-A5EFF0351BF4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D28E9E8-0760-44F5-8D1F-677C940DD9A6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5364396A-C179-4798-AB10-171C8F488944}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59CF13BC-96EF-46D6-B982-A0CD67FE4D2D}"/>
 </file>
</xml_diff>